<commit_message>
Coordination sheet: carry Y1 lesson-plan links into 2026-27 syllabus column
Fixes blue/underline styling that had been copied down the whole column
without links; only lessons with a plan Doc are linked now.

Claude-Session: https://claude.ai/code/session_016DNoLcEJU8JpjJFeZeoW28
</commit_message>
<xml_diff>
--- a/datalayer/rawdata/3B_Class_OLV_coordination_sheet.xlsx
+++ b/datalayer/rawdata/3B_Class_OLV_coordination_sheet.xlsx
@@ -94,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -171,6 +171,12 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -513,7 +519,7 @@
       <c r="D2" s="7" t="n"/>
       <c r="H2" s="23" t="inlineStr">
         <is>
-          <t>9/21/25 · Nick lead (lesson plan)</t>
+          <t>9/21/25 · Nick lead</t>
         </is>
       </c>
     </row>
@@ -530,7 +536,7 @@
       <c r="D3" s="7" t="n"/>
       <c r="H3" s="23" t="inlineStr">
         <is>
-          <t>9/28/25 (with Sess. 3) · Nick lead, Robb 2nd (lesson plan)</t>
+          <t>9/28/25 (with Sess. 3) · Nick lead, Robb 2nd</t>
         </is>
       </c>
     </row>
@@ -547,7 +553,7 @@
       <c r="D4" s="7" t="n"/>
       <c r="H4" s="23" t="inlineStr">
         <is>
-          <t>9/28/25 (with Sess. 2) · Nick lead, Robb 2nd (lesson plan)</t>
+          <t>9/28/25 (with Sess. 2) · Nick lead, Robb 2nd</t>
         </is>
       </c>
     </row>
@@ -560,7 +566,7 @@
           <t>No Class – Columbus Marathon</t>
         </is>
       </c>
-      <c r="C5" s="26" t="inlineStr">
+      <c r="C5" s="30" t="inlineStr">
         <is>
           <t>No class due to the Columbus Marathon</t>
         </is>
@@ -602,7 +608,7 @@
       <c r="D6" s="7" t="n"/>
       <c r="H6" s="23" t="inlineStr">
         <is>
-          <t>10/5/25 · Nick lead, Cristina 2nd (lesson plan)</t>
+          <t>10/5/25 · Nick lead, Cristina 2nd</t>
         </is>
       </c>
     </row>
@@ -611,7 +617,7 @@
         <v>46327</v>
       </c>
       <c r="B7" s="5" t="n"/>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="31" t="inlineStr">
         <is>
           <t>All Saints and All Souls pgs. 237–240 / All Saints Celebration in class – 4th graders present Saints / Donuts / Hand out Christmas Pageant scripts, go over lines if time allows</t>
         </is>
@@ -628,7 +634,7 @@
         <v>46334</v>
       </c>
       <c r="B8" s="5" t="n"/>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="31" t="inlineStr">
         <is>
           <t>Session 10 Celebrating Advent pgs. 79–84 / Send home Advent calendars (special place to follow during Advent) / Practice lines with the other 3rd grade class</t>
         </is>
@@ -645,7 +651,7 @@
         <v>46341</v>
       </c>
       <c r="B9" s="5" t="n"/>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="31" t="inlineStr">
         <is>
           <t>Session 14 Mary is Holy pgs. 113–120 / Rehearse in class together</t>
         </is>
@@ -662,7 +668,7 @@
         <v>46348</v>
       </c>
       <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="31" t="inlineStr">
         <is>
           <t>Session 15 Celebrating Christmas pgs. 121–126 / Rehearse in class together</t>
         </is>
@@ -683,7 +689,7 @@
           <t>No Class – Thanksgiving</t>
         </is>
       </c>
-      <c r="C11" s="26" t="inlineStr">
+      <c r="C11" s="30" t="inlineStr">
         <is>
           <t>No class due to Thanksgiving</t>
         </is>
@@ -721,7 +727,7 @@
           <t>Christmas Play</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="31" t="inlineStr">
         <is>
           <t>Christmas Play – Arrive at 8:30 am / Bagels in classroom / Send home St. Nicholas gifts with students</t>
         </is>
@@ -742,7 +748,7 @@
           <t>No Class – Christmas Break</t>
         </is>
       </c>
-      <c r="C13" s="26" t="inlineStr">
+      <c r="C13" s="30" t="inlineStr">
         <is>
           <t>No class due to Christmas break</t>
         </is>
@@ -780,7 +786,7 @@
           <t>No Class – Christmas Break</t>
         </is>
       </c>
-      <c r="C14" s="26" t="inlineStr">
+      <c r="C14" s="30" t="inlineStr">
         <is>
           <t>No class due to Christmas break</t>
         </is>
@@ -818,7 +824,7 @@
           <t>No Class – Christmas Break</t>
         </is>
       </c>
-      <c r="C15" s="26" t="inlineStr">
+      <c r="C15" s="30" t="inlineStr">
         <is>
           <t>No class due to Christmas break</t>
         </is>
@@ -856,7 +862,7 @@
           <t>No Class – Christmas Break</t>
         </is>
       </c>
-      <c r="C16" s="26" t="inlineStr">
+      <c r="C16" s="30" t="inlineStr">
         <is>
           <t>No class due to Christmas break</t>
         </is>
@@ -890,7 +896,7 @@
         <v>46397</v>
       </c>
       <c r="B17" s="5" t="n"/>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="31" t="inlineStr">
         <is>
           <t>Baptism of the Lord – Deacon Rob talks to students in groups about baptism / Session 16 Sacraments of Initiation pgs. 131–138 / Blessing of the Chalk – Deacon Rob blesses; bag chalk with the prayer to send home</t>
         </is>
@@ -911,7 +917,7 @@
           <t>No Class – Holiday Weekend</t>
         </is>
       </c>
-      <c r="C18" s="26" t="inlineStr">
+      <c r="C18" s="30" t="inlineStr">
         <is>
           <t>No class due to holiday weekend</t>
         </is>
@@ -945,7 +951,7 @@
         <v>46411</v>
       </c>
       <c r="B19" s="5" t="n"/>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="31" t="inlineStr">
         <is>
           <t>Session 18 Celebrating Jesus pgs. 147–154 / Celebrating the Lord's Day pgs. 254–259</t>
         </is>
@@ -962,7 +968,7 @@
         <v>46418</v>
       </c>
       <c r="B20" s="5" t="n"/>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="31" t="inlineStr">
         <is>
           <t>Session 17 Celebrating Reconciliation pgs. 139–145 / Session 22 Making Good Choices pgs. 181–188 / Prep for Reconciliation next weekend</t>
         </is>
@@ -983,7 +989,7 @@
           <t>3rd Gr Reconciliation 9:05am in Church</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="31" t="inlineStr">
         <is>
           <t>Reconciliation in the Church 9:05 am – head over right after morning prayer (3 priests; Krissy Murray leads the service with the priest) / The Bible and You pgs. 243-243 (likely 242–243) – have them look up scripture</t>
         </is>
@@ -1004,7 +1010,7 @@
           <t>No Class – Holiday Weekend</t>
         </is>
       </c>
-      <c r="C22" s="26" t="inlineStr">
+      <c r="C22" s="30" t="inlineStr">
         <is>
           <t>No class due to holiday weekend</t>
         </is>
@@ -1038,7 +1044,7 @@
         <v>46439</v>
       </c>
       <c r="B23" s="5" t="n"/>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="31" t="inlineStr">
         <is>
           <t>Session 20 Celebrating Lent and Holy Week pgs. 162–168 / Lent pgs. 221–224</t>
         </is>
@@ -1055,7 +1061,7 @@
         <v>46446</v>
       </c>
       <c r="B24" s="5" t="n"/>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" s="31" t="inlineStr">
         <is>
           <t>Session 8 Jesus Gathers Disciples pgs. 63–70 / Session 23 Living As God's Children pgs. 189–196</t>
         </is>
@@ -1076,7 +1082,7 @@
           <t>No Class – Irish Breakfast</t>
         </is>
       </c>
-      <c r="C25" s="26" t="inlineStr">
+      <c r="C25" s="30" t="inlineStr">
         <is>
           <t>No class due to the Irish Breakfast</t>
         </is>
@@ -1110,7 +1116,7 @@
         <v>46460</v>
       </c>
       <c r="B26" s="5" t="n"/>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C26" s="31" t="inlineStr">
         <is>
           <t>Session 25 Celebrating Easter pgs. 205–210 / The Last Supper pgs. 148, 153, 154, 225, 272 / Session 9 Jesus Rises from the Dead pgs. 71–78</t>
         </is>
@@ -1131,7 +1137,7 @@
           <t>No Class – Spring Break</t>
         </is>
       </c>
-      <c r="C27" s="26" t="inlineStr">
+      <c r="C27" s="30" t="inlineStr">
         <is>
           <t>No class due to spring breaks and Easter Sunday</t>
         </is>
@@ -1169,7 +1175,7 @@
           <t>No Class – Easter</t>
         </is>
       </c>
-      <c r="C28" s="26" t="inlineStr">
+      <c r="C28" s="30" t="inlineStr">
         <is>
           <t>No class due to spring breaks and Easter Sunday</t>
         </is>
@@ -1207,7 +1213,7 @@
           <t>No Class – Spring Break</t>
         </is>
       </c>
-      <c r="C29" s="26" t="inlineStr">
+      <c r="C29" s="30" t="inlineStr">
         <is>
           <t>No class due to spring breaks and Easter Sunday</t>
         </is>
@@ -1241,7 +1247,7 @@
         <v>46488</v>
       </c>
       <c r="B30" s="5" t="n"/>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" s="31" t="inlineStr">
         <is>
           <t>All Life is Sacred pgs. 197–204 (Session 24)</t>
         </is>
@@ -1258,7 +1264,7 @@
         <v>46495</v>
       </c>
       <c r="B31" s="5" t="n"/>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" s="31" t="inlineStr">
         <is>
           <t>Session 12 Jesus Sends the Holy Spirit pgs. 97–104 (last year: Session 11, pgs. 89–96 – confirm) / Pentecost pgs. 233–236</t>
         </is>
@@ -1279,7 +1285,7 @@
           <t>Last Class</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C32" s="31" t="inlineStr">
         <is>
           <t>Last day of class / Have fun in the classroom / Collect non-perishable food for Heart-to-Heart Food Pantry</t>
         </is>
@@ -1294,169 +1300,169 @@
     <row r="33" ht="15.75" customHeight="1" s="22">
       <c r="A33" s="4" t="n"/>
       <c r="B33" s="5" t="n"/>
-      <c r="C33" s="6" t="n"/>
+      <c r="C33" s="31" t="n"/>
       <c r="D33" s="7" t="n"/>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="22">
       <c r="A34" s="4" t="n"/>
       <c r="B34" s="5" t="n"/>
-      <c r="C34" s="6" t="n"/>
+      <c r="C34" s="31" t="n"/>
       <c r="D34" s="7" t="n"/>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="22">
       <c r="A35" s="4" t="n"/>
       <c r="B35" s="5" t="n"/>
-      <c r="C35" s="6" t="n"/>
+      <c r="C35" s="31" t="n"/>
       <c r="D35" s="7" t="n"/>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="22">
       <c r="A36" s="4" t="n"/>
       <c r="B36" s="5" t="n"/>
-      <c r="C36" s="6" t="n"/>
+      <c r="C36" s="31" t="n"/>
       <c r="D36" s="7" t="n"/>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="22">
       <c r="A37" s="4" t="n"/>
       <c r="B37" s="5" t="n"/>
-      <c r="C37" s="6" t="n"/>
+      <c r="C37" s="31" t="n"/>
       <c r="D37" s="7" t="n"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="22">
       <c r="A38" s="4" t="n"/>
       <c r="B38" s="5" t="n"/>
-      <c r="C38" s="6" t="n"/>
+      <c r="C38" s="31" t="n"/>
       <c r="D38" s="7" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="22">
       <c r="A39" s="4" t="n"/>
       <c r="B39" s="5" t="n"/>
-      <c r="C39" s="6" t="n"/>
+      <c r="C39" s="31" t="n"/>
       <c r="D39" s="7" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="22">
       <c r="A40" s="4" t="n"/>
       <c r="B40" s="5" t="n"/>
-      <c r="C40" s="6" t="n"/>
+      <c r="C40" s="31" t="n"/>
       <c r="D40" s="7" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="22">
       <c r="A41" s="4" t="n"/>
       <c r="B41" s="5" t="n"/>
-      <c r="C41" s="6" t="n"/>
+      <c r="C41" s="31" t="n"/>
       <c r="D41" s="7" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="22">
       <c r="A42" s="4" t="n"/>
       <c r="B42" s="5" t="n"/>
-      <c r="C42" s="6" t="n"/>
+      <c r="C42" s="31" t="n"/>
       <c r="D42" s="7" t="n"/>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="22">
       <c r="A43" s="4" t="n"/>
       <c r="B43" s="5" t="n"/>
-      <c r="C43" s="6" t="n"/>
+      <c r="C43" s="31" t="n"/>
       <c r="D43" s="7" t="n"/>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="22">
       <c r="A44" s="4" t="n"/>
       <c r="B44" s="5" t="n"/>
-      <c r="C44" s="6" t="n"/>
+      <c r="C44" s="31" t="n"/>
       <c r="D44" s="7" t="n"/>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="22">
       <c r="A45" s="4" t="n"/>
       <c r="B45" s="5" t="n"/>
-      <c r="C45" s="6" t="n"/>
+      <c r="C45" s="31" t="n"/>
       <c r="D45" s="7" t="n"/>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="22">
       <c r="A46" s="4" t="n"/>
       <c r="B46" s="5" t="n"/>
-      <c r="C46" s="6" t="n"/>
+      <c r="C46" s="31" t="n"/>
       <c r="D46" s="7" t="n"/>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="22">
       <c r="A47" s="4" t="n"/>
       <c r="B47" s="5" t="n"/>
-      <c r="C47" s="6" t="n"/>
+      <c r="C47" s="31" t="n"/>
       <c r="D47" s="7" t="n"/>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="22">
       <c r="A48" s="4" t="n"/>
       <c r="B48" s="5" t="n"/>
-      <c r="C48" s="6" t="n"/>
+      <c r="C48" s="31" t="n"/>
       <c r="D48" s="7" t="n"/>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="22">
       <c r="A49" s="4" t="n"/>
       <c r="B49" s="5" t="n"/>
-      <c r="C49" s="6" t="n"/>
+      <c r="C49" s="31" t="n"/>
       <c r="D49" s="7" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="22">
       <c r="A50" s="4" t="n"/>
       <c r="B50" s="5" t="n"/>
-      <c r="C50" s="6" t="n"/>
+      <c r="C50" s="31" t="n"/>
       <c r="D50" s="7" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="22">
       <c r="A51" s="4" t="n"/>
       <c r="B51" s="5" t="n"/>
-      <c r="C51" s="6" t="n"/>
+      <c r="C51" s="31" t="n"/>
       <c r="D51" s="7" t="n"/>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="22">
       <c r="A52" s="4" t="n"/>
       <c r="B52" s="5" t="n"/>
-      <c r="C52" s="6" t="n"/>
+      <c r="C52" s="31" t="n"/>
       <c r="D52" s="7" t="n"/>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="22">
       <c r="A53" s="4" t="n"/>
       <c r="B53" s="5" t="n"/>
-      <c r="C53" s="6" t="n"/>
+      <c r="C53" s="31" t="n"/>
       <c r="D53" s="7" t="n"/>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="22">
       <c r="A54" s="4" t="n"/>
       <c r="B54" s="5" t="n"/>
-      <c r="C54" s="6" t="n"/>
+      <c r="C54" s="31" t="n"/>
       <c r="D54" s="7" t="n"/>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="22">
       <c r="A55" s="4" t="n"/>
       <c r="B55" s="5" t="n"/>
-      <c r="C55" s="6" t="n"/>
+      <c r="C55" s="31" t="n"/>
       <c r="D55" s="7" t="n"/>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="22">
       <c r="A56" s="4" t="n"/>
       <c r="B56" s="5" t="n"/>
-      <c r="C56" s="6" t="n"/>
+      <c r="C56" s="31" t="n"/>
       <c r="D56" s="7" t="n"/>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="22">
       <c r="A57" s="4" t="n"/>
       <c r="B57" s="5" t="n"/>
-      <c r="C57" s="6" t="n"/>
+      <c r="C57" s="31" t="n"/>
       <c r="D57" s="7" t="n"/>
     </row>
     <row r="58" ht="15.75" customHeight="1" s="22">
       <c r="A58" s="4" t="n"/>
       <c r="B58" s="5" t="n"/>
-      <c r="C58" s="6" t="n"/>
+      <c r="C58" s="31" t="n"/>
       <c r="D58" s="7" t="n"/>
     </row>
     <row r="59" ht="15.75" customHeight="1" s="22">
       <c r="A59" s="4" t="n"/>
       <c r="B59" s="5" t="n"/>
-      <c r="C59" s="6" t="n"/>
+      <c r="C59" s="31" t="n"/>
       <c r="D59" s="7" t="n"/>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="22">
       <c r="A60" s="4" t="n"/>
       <c r="B60" s="5" t="n"/>
-      <c r="C60" s="6" t="n"/>
+      <c r="C60" s="31" t="n"/>
       <c r="D60" s="7" t="n"/>
     </row>
     <row r="61" ht="15.75" customHeight="1" s="22">
@@ -6156,10 +6162,10 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" scale="70"/>

</xml_diff>

<commit_message>
Y1 coloring-sheet inventory: 13 files, Drive folder, sheet column
- Found coloring pages in Downloads by date added; uploaded to
  3rdgradeOLV/Coloring Sheets (personal Drive) and copied to rawdata/coloring
- Added linked 'Coloring sheet' column to the 2025-26 tab
- coloring_sheets.md index; Session 16/20 note Docs exported
- CLAUDE.md: Drive folder ids, reuse map notes coloring per session

Claude-Session: https://claude.ai/code/session_016DNoLcEJU8JpjJFeZeoW28
</commit_message>
<xml_diff>
--- a/datalayer/rawdata/3B_Class_OLV_coordination_sheet.xlsx
+++ b/datalayer/rawdata/3B_Class_OLV_coordination_sheet.xlsx
@@ -94,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -178,6 +178,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6185,7 +6188,7 @@
     <col width="29.86" customWidth="1" style="22" min="2" max="2"/>
     <col width="40" customWidth="1" style="22" min="3" max="3"/>
     <col width="12.43" customWidth="1" style="22" min="4" max="7"/>
-    <col width="8.710000000000001" customWidth="1" style="22" min="8" max="26"/>
+    <col width="34" customWidth="1" style="22" min="8" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6224,6 +6227,11 @@
           <t>Chad</t>
         </is>
       </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Coloring sheet</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
@@ -6244,6 +6252,11 @@
           <t>Lead</t>
         </is>
       </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>St. Ignatius Loyola</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -6269,6 +6282,11 @@
           <t>2nd</t>
         </is>
       </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Holy Trinity stained glass (+ unlabeled version in folder)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -6294,6 +6312,11 @@
           <t>2nd</t>
         </is>
       </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Angel appears to Joseph</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -6407,6 +6430,11 @@
       <c r="G8" s="7" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="H8" s="32" t="inlineStr">
+        <is>
+          <t>Miraculous Medal</t>
         </is>
       </c>
     </row>
@@ -6836,7 +6864,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="H21" s="20" t="n"/>
+      <c r="H21" s="32" t="inlineStr">
+        <is>
+          <t>Gifts of the Holy Spirit toolbox (+ blank version in folder)</t>
+        </is>
+      </c>
       <c r="I21" s="20" t="n"/>
       <c r="J21" s="20" t="n"/>
       <c r="K21" s="20" t="n"/>
@@ -7020,7 +7052,11 @@
         </is>
       </c>
       <c r="G25" s="19" t="n"/>
-      <c r="H25" s="20" t="n"/>
+      <c r="H25" s="32" t="inlineStr">
+        <is>
+          <t>Jesus and the Woman at the Well</t>
+        </is>
+      </c>
       <c r="I25" s="20" t="n"/>
       <c r="J25" s="20" t="n"/>
       <c r="K25" s="20" t="n"/>
@@ -7104,7 +7140,11 @@
         </is>
       </c>
       <c r="G27" s="20" t="n"/>
-      <c r="H27" s="20" t="n"/>
+      <c r="H27" s="32" t="inlineStr">
+        <is>
+          <t>St. Carlo Acutis – Eucharist is my highway to heaven</t>
+        </is>
+      </c>
       <c r="I27" s="20" t="n"/>
       <c r="J27" s="20" t="n"/>
       <c r="K27" s="20" t="n"/>
@@ -7150,7 +7190,11 @@
         </is>
       </c>
       <c r="G28" s="20" t="n"/>
-      <c r="H28" s="20" t="n"/>
+      <c r="H28" s="32" t="inlineStr">
+        <is>
+          <t>Stations of the Cross</t>
+        </is>
+      </c>
       <c r="I28" s="20" t="n"/>
       <c r="J28" s="20" t="n"/>
       <c r="K28" s="20" t="n"/>
@@ -7225,7 +7269,11 @@
         </is>
       </c>
       <c r="F30" s="20" t="n"/>
-      <c r="H30" s="20" t="n"/>
+      <c r="H30" s="32" t="inlineStr">
+        <is>
+          <t>Alleluia! Jesus is Risen (+ Alleluia lamb in folder)</t>
+        </is>
+      </c>
       <c r="I30" s="20" t="n"/>
       <c r="J30" s="20" t="n"/>
       <c r="K30" s="20" t="n"/>
@@ -7495,7 +7543,11 @@
       <c r="E37" s="20" t="n"/>
       <c r="F37" s="20" t="n"/>
       <c r="G37" s="20" t="n"/>
-      <c r="H37" s="20" t="n"/>
+      <c r="H37" s="32" t="inlineStr">
+        <is>
+          <t>Holy Spirit dove stained glass (+ Gifts of the Holy Spirit toolbox reused)</t>
+        </is>
+      </c>
       <c r="I37" s="20" t="n"/>
       <c r="J37" s="20" t="n"/>
       <c r="K37" s="20" t="n"/>
@@ -12497,8 +12549,18 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" scale="70"/>

</xml_diff>